<commit_message>
Leila Identity kart görselleri + Prism Core implementasyonu + temizlik
- Leila Identity kartlarının tüm görselleri eklendi (14 kart)
- Prism Core: orbit'teyken 2s'de bir 55px içindeki düşmanlara rastgele element uygular
- Prism Core min_level 3 → 2, açıklaması güncellendi
- Steam Core açıklaması gerçek implementasyona göre güncellendi (Türkçe)
- Tempest Core ve Prismatic Core dead code kaldırıldı (ball.gd)
- leilaCards.xlsx: Tempest/Prismatic Core silindi, Steam/Prism Core açıklamaları güncellendi
- mistCore görselleri güncellendi
- anchor_core_art.png güncellendi

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/leilaCards.xlsx
+++ b/leilaCards.xlsx
@@ -543,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -762,12 +762,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Hits Wet targets → small AoE burst</t>
+          <t>Leaves a steam cloud on hit. Applies Wet to nearby enemies after 0.8s</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Islak + Yanan → Buhar patlaması</t>
+          <t>Carptiği noktada buhar bulutu birakir, Yakindaki dusmanlara Wet uygular</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Stays in orbit, applies random element to nearby enemies</t>
+          <t>Stays in orbit. Applies random element to nearby enemies every 2s</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Orbit'te kalir, yakin dusmanlaara rastgele element uygular</t>
+          <t>Orbit'te kalir, yakin dusmanlara rastgele element uygular (her 2s)</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -912,70 +912,70 @@
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Tempest Core</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Kimlik</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Changes to a random Element | after each wall bounce</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Fırtına alanı oluşturur</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>Epik</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>-- Yardimci (Utility) --</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Prismatic Core</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Kimlik</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Randomly changes Element | after every enemy hit</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Her sekmede element değiştirir</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>Ender</t>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Electric Amp</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Yardimci</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Electric Core +2 damage</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Yaygin</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>-- Yardimci (Utility) --</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Cryo Amp</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Yardimci</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Cryo Core +2 damage</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Yaygin</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Electric Amp</t>
+          <t>Hydro Amp</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Electric Core +2 damage</t>
+          <t>Hydro Core +2 damage</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Cryo Amp</t>
+          <t>Pyro Amp</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Cryo Core +2 damage</t>
+          <t>Pyro Core +2 damage</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1029,7 +1029,7 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Hydro Amp</t>
+          <t>Conduction</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Hydro Core +2 damage</t>
+          <t>Electric reaction range +30%</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1047,16 +1047,16 @@
           <t>---</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Yaygin</t>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Nadir</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Pyro Amp</t>
+          <t>Hydro Pressure</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Pyro Core +2 damage</t>
+          <t>Wet-applying Cores orbit faster</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -1074,16 +1074,16 @@
           <t>---</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>Yaygin</t>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Nadir</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Conduction</t>
+          <t>Arc Amplifier</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Electric reaction range +30%</t>
+          <t>Arc Core +1 düşmana daha yayar</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1110,7 +1110,7 @@
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Hydro Pressure</t>
+          <t>Static Charge</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Wet-applying Cores orbit faster</t>
+          <t>Electrified enemies transfer damage | to each other</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -1137,7 +1137,7 @@
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Arc Amplifier</t>
+          <t>Supercooling</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Arc Core +1 düşmana daha yayar</t>
+          <t>Cryo enemies slowed further</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1164,7 +1164,7 @@
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Static Charge</t>
+          <t>Thermal Vision</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Electrified enemies transfer damage | to each other</t>
+          <t>Burning enemies take more damage</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -1191,7 +1191,7 @@
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Supercooling</t>
+          <t>Living Storm</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Cryo enemies slowed further</t>
+          <t>Electrified enemies approaching you | trigger small lightning</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1218,7 +1218,7 @@
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Thermal Vision</t>
+          <t>Arcane Mind</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Burning enemies take more damage</t>
+          <t>First applied element lasts 100% longer</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1236,16 +1236,16 @@
           <t>---</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>Nadir</t>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Ender</t>
         </is>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Living Storm</t>
+          <t>Frozen Time</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1255,24 +1255,24 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Electrified enemies approaching you | trigger small lightning</t>
+          <t>Freeze duration +30%</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>Nadir</t>
+          <t>Donuk düşmana isabet → donma yenilenir</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Ender</t>
         </is>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Arcane Mind</t>
+          <t>Overheat</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>First applied element lasts 100% longer</t>
+          <t>Burn explodes after 7 stacks</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -1299,7 +1299,7 @@
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Frozen Time</t>
+          <t>Elemental Harmony</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Freeze duration +30%</t>
+          <t>Per unique active element: | +5% Core Speed</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Donuk düşmana isabet → donma yenilenir</t>
+          <t>2 farklı element aktifse Core hızı +%10</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -1326,7 +1326,7 @@
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Overheat</t>
+          <t>Resonance Engine</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Burn explodes after 7 stacks</t>
+          <t>Each Reaction → +1 Momentum | Each Momentum → +3% Core Speed</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -1353,7 +1353,7 @@
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Elemental Harmony</t>
+          <t>Pyroblast</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1363,12 +1363,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Per unique active element: | +5% Core Speed</t>
+          <t>Burn explosions gain Area | based on Burn Stacks</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>2 farklı element aktifse Core hızı +%10</t>
+          <t>Yanan düşmana critical → patlama</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -1380,7 +1380,7 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Resonance Engine</t>
+          <t>Thermal Expansion</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1390,24 +1390,24 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Each Reaction → +1 Momentum | Each Momentum → +3% Core Speed</t>
+          <t>Steam explosion area grows</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
-        <is>
-          <t>Ender</t>
+          <t>Yangın yığınları daha hızlı birikir</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>Epik</t>
         </is>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Pyroblast</t>
+          <t>Mana Overflow</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1417,24 +1417,24 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Burn explosions gain Area | based on Burn Stacks</t>
+          <t>Using Calamity empowers | all Cores briefly</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Yanan düşmana critical → patlama</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>Ender</t>
+          <t>Max element kapasitesi +1</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>Epik</t>
         </is>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Thermal Expansion</t>
+          <t>Perfect Catalyst</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1444,12 +1444,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Steam explosion area grows</t>
+          <t>Reaction → reapply last used element</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Yangın yığınları daha hızlı birikir</t>
+          <t>Reaksiyon → ek ateşleme uygular</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
@@ -1461,7 +1461,7 @@
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Mana Overflow</t>
+          <t>Chain Catalyst</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1471,24 +1471,24 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Using Calamity empowers | all Cores briefly</t>
+          <t>2+ elements on target: | Reactions deal +30% dmg</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Max element kapasitesi +1</t>
-        </is>
-      </c>
-      <c r="E36" s="12" t="inlineStr">
-        <is>
-          <t>Epik</t>
+          <t>2+ element → +%30 reaksiyon hasarı</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Nadir</t>
         </is>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Perfect Catalyst</t>
+          <t>Core Mastery</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1498,85 +1498,85 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Reaction → reapply last used element</t>
+          <t>+1 damage to all cores</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Reaksiyon → ek ateşleme uygular</t>
-        </is>
-      </c>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>Epik</t>
+          <t>Tüm core'lara +1 hasar</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Yaygin</t>
         </is>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>Chain Catalyst</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Yardimci</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>2+ elements on target: | Reactions deal +30% dmg</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>2+ element → +%30 reaksiyon hasarı</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>Nadir</t>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>-- Bireysellik (Individuality) --</t>
         </is>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Core Mastery</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Yardimci</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>+1 damage to all cores</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Tüm core'lara +1 hasar</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Speed Upgrade</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Bireysellik</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Movement speed increases</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Hareket hızı artar</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>Yaygin</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>-- Bireysellik (Individuality) --</t>
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Max Health Up</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Bireysellik</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Maximum HP +5</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Maksimum HP +5</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Yaygin</t>
         </is>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Speed Upgrade</t>
+          <t>Medkit</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1586,12 +1586,12 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Movement speed increases</t>
+          <t>+10 HP restored</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Hareket hızı artar</t>
+          <t>+10 HP iyileştirilir</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -1603,7 +1603,7 @@
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Max Health Up</t>
+          <t>Mystic Flow</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -1613,24 +1613,24 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Maximum HP +5</t>
+          <t>Each unique element applied | → +1% Move Speed (max 20%)</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Maksimum HP +5</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>Yaygin</t>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Nadir</t>
         </is>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Medkit</t>
+          <t>Elemental Memory</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1640,24 +1640,24 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>+10 HP restored</t>
+          <t>Reacted enemies hold new elements | 100% longer (4s)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>+10 HP iyileştirilir</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>Yaygin</t>
+          <t>Reaksiyon geçmişi → debuff süresi x2</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Nadir</t>
         </is>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Mystic Flow</t>
+          <t>Resonant Soul</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Each unique element applied | → +1% Move Speed (max 20%)</t>
+          <t>Each Reaction → restore 2 HP</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -1684,7 +1684,7 @@
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Elemental Memory</t>
+          <t>Catalyst Mind</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1694,24 +1694,24 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Reacted enemies hold new elements | 100% longer (4s)</t>
+          <t>After a Reaction, next element | applies twice (5s cooldown)</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Reaksiyon geçmişi → debuff süresi x2</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>Nadir</t>
+          <t>Reaksiyon sonrası 2s: tüm hasar +%15</t>
+        </is>
+      </c>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>Efsanevi</t>
         </is>
       </c>
     </row>
     <row r="46" ht="28" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Resonant Soul</t>
+          <t>Volatile Mixture</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -1721,85 +1721,85 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Each Reaction → restore 2 HP</t>
+          <t>3rd element on target: | instantly triggers Reaction</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Nadir</t>
+          <t>3. element → anında reaksiyon</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="inlineStr">
+        <is>
+          <t>Ender</t>
         </is>
       </c>
     </row>
     <row r="47" ht="28" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>Catalyst Mind</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>Bireysellik</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>After a Reaction, next element | applies twice (5s cooldown)</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>Reaksiyon sonrası 2s: tüm hasar +%15</t>
-        </is>
-      </c>
-      <c r="E47" s="13" t="inlineStr">
-        <is>
-          <t>Efsanevi</t>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>-- Felaket (Calamity) --</t>
         </is>
       </c>
     </row>
     <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>Volatile Mixture</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Bireysellik</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>3rd element on target: | instantly triggers Reaction</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>3. element → anında reaksiyon</t>
-        </is>
-      </c>
-      <c r="E48" s="10" t="inlineStr">
-        <is>
-          <t>Ender</t>
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Monsoon</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Felaket</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>All enemies in the Yard | gain Wet</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Sahada ki tüm düşmanlar ıslanır</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>Epik</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>-- Felaket (Calamity) --</t>
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>EMP Pulse</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Felaket</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>All Electrified enemies | in the Yard take 15 dmg</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Sahada ki Elektrikli düşmanlar 15 hasar alır</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>Epik</t>
         </is>
       </c>
     </row>
     <row r="50" ht="28" customHeight="1">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Monsoon</t>
+          <t>Blizzard</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1809,24 +1809,24 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>All enemies in the Yard | gain Wet</t>
+          <t>The entire Yard freezes | for 3s</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Sahada ki tüm düşmanlar ıslanır</t>
-        </is>
-      </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>Epik</t>
+          <t>Sahada ki tüm düşmanlar 3s donar</t>
+        </is>
+      </c>
+      <c r="E50" s="13" t="inlineStr">
+        <is>
+          <t>Efsanevi</t>
         </is>
       </c>
     </row>
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>EMP Pulse</t>
+          <t>Volcanic Rift</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -1836,24 +1836,24 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>All Electrified enemies | in the Yard take 15 dmg</t>
+          <t>Leaves lava trail on ground</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Sahada ki Elektrikli düşmanlar 15 hasar alır</t>
-        </is>
-      </c>
-      <c r="E51" s="11" t="inlineStr">
-        <is>
-          <t>Epik</t>
+          <t>Yerde lav izi bırakır</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>Efsanevi</t>
         </is>
       </c>
     </row>
     <row r="52" ht="28" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Blizzard</t>
+          <t>Thunderstorm</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>The entire Yard freezes | for 3s</t>
+          <t>Random lightning strikes for 5s</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Sahada ki tüm düşmanlar 3s donar</t>
+          <t>5s boyunca rastgele yıldırım düşer</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -1880,7 +1880,7 @@
     <row r="53" ht="28" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>Volcanic Rift</t>
+          <t>Lightning</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -1890,24 +1890,24 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Leaves lava trail on ground</t>
+          <t>Lightning strikes selected point</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Yerde lav izi bırakır</t>
-        </is>
-      </c>
-      <c r="E53" s="14" t="inlineStr">
-        <is>
-          <t>Efsanevi</t>
+          <t>Seçilen noktaya yıldırım düşer</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>Yaygin</t>
         </is>
       </c>
     </row>
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Thunderstorm</t>
+          <t>Flame Zone</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1917,78 +1917,78 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Random lightning strikes for 5s</t>
+          <t>Continuous damage in selected area</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>5s boyunca rastgele yıldırım düşer</t>
-        </is>
-      </c>
-      <c r="E54" s="13" t="inlineStr">
-        <is>
-          <t>Efsanevi</t>
+          <t>Seçilen alanda sürekli hasar</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Yaygin</t>
         </is>
       </c>
     </row>
     <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Lightning</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Felaket</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Lightning strikes selected point</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Seçilen noktaya yıldırım düşer</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>Yaygin</t>
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>Mist Core</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>Every 4s: applies Wet to 1 random enemy within 70px</t>
+        </is>
+      </c>
+      <c r="D55" s="15" t="inlineStr">
+        <is>
+          <t>Her 4s: 70px icerisinde 1 rastgele dusmana Islatma uygular</t>
+        </is>
+      </c>
+      <c r="E55" s="15" t="inlineStr">
+        <is>
+          <t>Nadiren Gorulen</t>
         </is>
       </c>
     </row>
     <row r="56" ht="28" customHeight="1">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>Flame Zone</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>Felaket</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>Continuous damage in selected area</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>Seçilen alanda sürekli hasar</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>Yaygin</t>
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>Frost Aura Core</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>Enemies entering 50px range automatically get Slowed</t>
+        </is>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>50px menzile giren dusmanlar otomatik Yavastir alir</t>
+        </is>
+      </c>
+      <c r="E56" s="15" t="inlineStr">
+        <is>
+          <t>Ender</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="15" t="inlineStr">
         <is>
-          <t>Mist Core</t>
+          <t>Static Aura Core</t>
         </is>
       </c>
       <c r="B57" s="15" t="inlineStr">
@@ -1998,24 +1998,24 @@
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>Every 4s: applies Wet to 1 random enemy within 70px</t>
+          <t>Enemies entering 60px range get Electrified (3s cooldown/enemy)</t>
         </is>
       </c>
       <c r="D57" s="15" t="inlineStr">
         <is>
-          <t>Her 4s: 70px icerisinde 1 rastgele dusmana Islatma uygular</t>
+          <t>60px menzile giren dusmanlar Elektriflenir (3s CD/dusman)</t>
         </is>
       </c>
       <c r="E57" s="15" t="inlineStr">
         <is>
-          <t>Nadiren Gorulen</t>
+          <t>Ender</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="15" t="inlineStr">
         <is>
-          <t>Frost Aura Core</t>
+          <t>Catalyst Pulse Core</t>
         </is>
       </c>
       <c r="B58" s="15" t="inlineStr">
@@ -2025,12 +2025,12 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Enemies entering 50px range automatically get Slowed</t>
+          <t>Every 5s: extends debuff durations on enemies within 120px by +1s</t>
         </is>
       </c>
       <c r="D58" s="15" t="inlineStr">
         <is>
-          <t>50px menzile giren dusmanlar otomatik Yavastir alir</t>
+          <t>Her 5s: 120px icerisindeki debufflu dusmanların surelerini +1s uzatir</t>
         </is>
       </c>
       <c r="E58" s="15" t="inlineStr">
@@ -2042,7 +2042,7 @@
     <row r="59">
       <c r="A59" s="15" t="inlineStr">
         <is>
-          <t>Static Aura Core</t>
+          <t>Echo Resonance Core</t>
         </is>
       </c>
       <c r="B59" s="15" t="inlineStr">
@@ -2052,24 +2052,24 @@
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>Enemies entering 60px range get Electrified (3s cooldown/enemy)</t>
+          <t>Every 5s: for 1s pulses last applied element to enemies within 80px</t>
         </is>
       </c>
       <c r="D59" s="15" t="inlineStr">
         <is>
-          <t>60px menzile giren dusmanlar Elektriflenir (3s CD/dusman)</t>
+          <t>Her 5s: 1s boyunca 80px icerisine son uygulanan elementi yayar</t>
         </is>
       </c>
       <c r="E59" s="15" t="inlineStr">
         <is>
-          <t>Ender</t>
+          <t>Destansı</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="15" t="inlineStr">
         <is>
-          <t>Catalyst Pulse Core</t>
+          <t>Volatile Aura Core</t>
         </is>
       </c>
       <c r="B60" s="15" t="inlineStr">
@@ -2079,24 +2079,24 @@
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>Every 5s: extends debuff durations on enemies within 120px by +1s</t>
+          <t>On reaction trigger: deals 2 damage pulse to enemies within 80px</t>
         </is>
       </c>
       <c r="D60" s="15" t="inlineStr">
         <is>
-          <t>Her 5s: 120px icerisindeki debufflu dusmanların surelerini +1s uzatir</t>
+          <t>Reaksiyon tetiklenince: 80px icerisine 2 hasar pulse atar</t>
         </is>
       </c>
       <c r="E60" s="15" t="inlineStr">
         <is>
-          <t>Ender</t>
+          <t>Destansı</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="15" t="inlineStr">
         <is>
-          <t>Echo Resonance Core</t>
+          <t>Elemental Shield Core</t>
         </is>
       </c>
       <c r="B61" s="15" t="inlineStr">
@@ -2106,78 +2106,78 @@
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>Every 5s: for 1s pulses last applied element to enemies within 80px</t>
+          <t>Last applied element grants 20%% resistance to that elements damage</t>
         </is>
       </c>
       <c r="D61" s="15" t="inlineStr">
         <is>
-          <t>Her 5s: 1s boyunca 80px icerisine son uygulanan elementi yayar</t>
+          <t>Son uygulanan element, o elementin hasarina karsi %%20 direnc saglar</t>
         </is>
       </c>
       <c r="E61" s="15" t="inlineStr">
         <is>
-          <t>Destansı</t>
+          <t>Ender</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="15" t="inlineStr">
         <is>
-          <t>Volatile Aura Core</t>
+          <t>Wet Armor</t>
         </is>
       </c>
       <c r="B62" s="15" t="inlineStr">
         <is>
-          <t>Kimlik</t>
+          <t>Bireysellik</t>
         </is>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>On reaction trigger: deals 2 damage pulse to enemies within 80px</t>
+          <t>While a Wet enemy exists in the Yard: take 10%% less damage</t>
         </is>
       </c>
       <c r="D62" s="15" t="inlineStr">
         <is>
-          <t>Reaksiyon tetiklenince: 80px icerisine 2 hasar pulse atar</t>
+          <t>Islak dusman varken %%10 az hasar alirsin</t>
         </is>
       </c>
       <c r="E62" s="15" t="inlineStr">
         <is>
-          <t>Destansı</t>
+          <t>Nadiren Gorulen</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="15" t="inlineStr">
         <is>
-          <t>Elemental Shield Core</t>
+          <t>Burn Frenzy</t>
         </is>
       </c>
       <c r="B63" s="15" t="inlineStr">
         <is>
-          <t>Kimlik</t>
+          <t>Bireysellik</t>
         </is>
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>Last applied element grants 20%% resistance to that elements damage</t>
+          <t>Each Burning enemy in the Yard: +2%% Core Speed (max +14%%)</t>
         </is>
       </c>
       <c r="D63" s="15" t="inlineStr">
         <is>
-          <t>Son uygulanan element, o elementin hasarina karsi %%20 direnc saglar</t>
+          <t>Her Yanan dusman icin +2%% Core Hizi (maks +14%%)</t>
         </is>
       </c>
       <c r="E63" s="15" t="inlineStr">
         <is>
-          <t>Ender</t>
+          <t>Nadiren Gorulen</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="15" t="inlineStr">
         <is>
-          <t>Wet Armor</t>
+          <t>Steam Surge</t>
         </is>
       </c>
       <c r="B64" s="15" t="inlineStr">
@@ -2187,12 +2187,12 @@
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>While a Wet enemy exists in the Yard: take 10%% less damage</t>
+          <t>Steam reaction: +15%% movement speed for 3s</t>
         </is>
       </c>
       <c r="D64" s="15" t="inlineStr">
         <is>
-          <t>Islak dusman varken %%10 az hasar alirsin</t>
+          <t>Steam reaksiyonu: 3s boyunca +15%% hareket hizi</t>
         </is>
       </c>
       <c r="E64" s="15" t="inlineStr">
@@ -2204,7 +2204,7 @@
     <row r="65">
       <c r="A65" s="15" t="inlineStr">
         <is>
-          <t>Burn Frenzy</t>
+          <t>Shock Reflex</t>
         </is>
       </c>
       <c r="B65" s="15" t="inlineStr">
@@ -2214,12 +2214,12 @@
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>Each Burning enemy in the Yard: +2%% Core Speed (max +14%%)</t>
+          <t>Electrocute reaction: +8%% dodge chance for 3s</t>
         </is>
       </c>
       <c r="D65" s="15" t="inlineStr">
         <is>
-          <t>Her Yanan dusman icin +2%% Core Hizi (maks +14%%)</t>
+          <t>Electrocute reaksiyonu: 3s icin +8%% hasar kacınma</t>
         </is>
       </c>
       <c r="E65" s="15" t="inlineStr">
@@ -2231,7 +2231,7 @@
     <row r="66">
       <c r="A66" s="15" t="inlineStr">
         <is>
-          <t>Steam Surge</t>
+          <t>Frost Barrier</t>
         </is>
       </c>
       <c r="B66" s="15" t="inlineStr">
@@ -2241,24 +2241,24 @@
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>Steam reaction: +15%% movement speed for 3s</t>
+          <t>Freeze reaction: gain a 5-HP shield for 4s</t>
         </is>
       </c>
       <c r="D66" s="15" t="inlineStr">
         <is>
-          <t>Steam reaksiyonu: 3s boyunca +15%% hareket hizi</t>
+          <t>Freeze reaksiyonu: 4s suren 5 HP kalkan</t>
         </is>
       </c>
       <c r="E66" s="15" t="inlineStr">
         <is>
-          <t>Nadiren Gorulen</t>
+          <t>Ender</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="15" t="inlineStr">
         <is>
-          <t>Shock Reflex</t>
+          <t>Primal Instinct</t>
         </is>
       </c>
       <c r="B67" s="15" t="inlineStr">
@@ -2268,24 +2268,24 @@
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>Electrocute reaction: +8%% dodge chance for 3s</t>
+          <t>3 unique reactions in one wave: +10%% damage for 5s</t>
         </is>
       </c>
       <c r="D67" s="15" t="inlineStr">
         <is>
-          <t>Electrocute reaksiyonu: 3s icin +8%% hasar kacınma</t>
+          <t>Bir dalgada 3 farkli reaksiyon: 5s icin +10%% hasar</t>
         </is>
       </c>
       <c r="E67" s="15" t="inlineStr">
         <is>
-          <t>Nadiren Gorulen</t>
+          <t>Ender</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="15" t="inlineStr">
         <is>
-          <t>Frost Barrier</t>
+          <t>Melt Spiral</t>
         </is>
       </c>
       <c r="B68" s="15" t="inlineStr">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>Freeze reaction: gain a 5-HP shield for 4s</t>
+          <t>Melt reaction: leave a 2s burning puddle on the enemy location (1 dmg/s)</t>
         </is>
       </c>
       <c r="D68" s="15" t="inlineStr">
         <is>
-          <t>Freeze reaksiyonu: 4s suren 5 HP kalkan</t>
+          <t>Melt reaksiyonu: dusmanin konumunda 2s alev birakir (1/s)</t>
         </is>
       </c>
       <c r="E68" s="15" t="inlineStr">
@@ -2312,7 +2312,7 @@
     <row r="69">
       <c r="A69" s="15" t="inlineStr">
         <is>
-          <t>Primal Instinct</t>
+          <t>Void Resonance</t>
         </is>
       </c>
       <c r="B69" s="15" t="inlineStr">
@@ -2322,39 +2322,39 @@
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>3 unique reactions in one wave: +10%% damage for 5s</t>
+          <t>4 unique reactions in one wave: next Calamity does not consume a slot</t>
         </is>
       </c>
       <c r="D69" s="15" t="inlineStr">
         <is>
-          <t>Bir dalgada 3 farkli reaksiyon: 5s icin +10%% hasar</t>
+          <t>Dalgada 4 farkli reaksiyon: sonraki Calamity slot tuketmez</t>
         </is>
       </c>
       <c r="E69" s="15" t="inlineStr">
         <is>
-          <t>Ender</t>
+          <t>Destansi</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="15" t="inlineStr">
         <is>
-          <t>Melt Spiral</t>
+          <t>Deep Freeze</t>
         </is>
       </c>
       <c r="B70" s="15" t="inlineStr">
         <is>
-          <t>Bireysellik</t>
+          <t>Felaket</t>
         </is>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Melt reaction: leave a 2s burning puddle on the enemy location (1 dmg/s)</t>
+          <t>Instantly Freezes all currently Wet enemies in the Yard</t>
         </is>
       </c>
       <c r="D70" s="15" t="inlineStr">
         <is>
-          <t>Melt reaksiyonu: dusmanin konumunda 2s alev birakir (1/s)</t>
+          <t>Tum Islak dusmanları anında Dondurur</t>
         </is>
       </c>
       <c r="E70" s="15" t="inlineStr">
@@ -2366,22 +2366,22 @@
     <row r="71">
       <c r="A71" s="15" t="inlineStr">
         <is>
-          <t>Void Resonance</t>
+          <t>Wildfire</t>
         </is>
       </c>
       <c r="B71" s="15" t="inlineStr">
         <is>
-          <t>Bireysellik</t>
+          <t>Felaket</t>
         </is>
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>4 unique reactions in one wave: next Calamity does not consume a slot</t>
+          <t>All Burning enemies explode: 10 damage, fire spreads to 2 nearby enemies</t>
         </is>
       </c>
       <c r="D71" s="15" t="inlineStr">
         <is>
-          <t>Dalgada 4 farkli reaksiyon: sonraki Calamity slot tuketmez</t>
+          <t>Tum Yanan dusmanlar patlar (10 hasar, 2 yakina yangin yayilir)</t>
         </is>
       </c>
       <c r="E71" s="15" t="inlineStr">
@@ -2393,22 +2393,22 @@
     <row r="72">
       <c r="A72" s="15" t="inlineStr">
         <is>
-          <t>Deep Freeze</t>
+          <t>Cryo Burst</t>
         </is>
       </c>
       <c r="B72" s="15" t="inlineStr">
         <is>
-          <t>Felaket</t>
+          <t>Yardimci</t>
         </is>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>Instantly Freezes all currently Wet enemies in the Yard</t>
+          <t>Slowed enemy: next hit deals +8 bonus damage</t>
         </is>
       </c>
       <c r="D72" s="15" t="inlineStr">
         <is>
-          <t>Tum Islak dusmanları anında Dondurur</t>
+          <t>Yavasslatilmis dusmana sonraki vurus +8 bonus hasar</t>
         </is>
       </c>
       <c r="E72" s="15" t="inlineStr">
@@ -2420,79 +2420,25 @@
     <row r="73">
       <c r="A73" s="15" t="inlineStr">
         <is>
-          <t>Wildfire</t>
+          <t>Arc Overload</t>
         </is>
       </c>
       <c r="B73" s="15" t="inlineStr">
         <is>
-          <t>Felaket</t>
+          <t>Yardimci</t>
         </is>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>All Burning enemies explode: 10 damage, fire spreads to 2 nearby enemies</t>
+          <t>Electrocute chain hits 2 additional enemies (5 damage each)</t>
         </is>
       </c>
       <c r="D73" s="15" t="inlineStr">
         <is>
-          <t>Tum Yanan dusmanlar patlar (10 hasar, 2 yakina yangin yayilir)</t>
+          <t>Electrocute zinciri 2 ek dusmana daha sicrar (5 hasar)</t>
         </is>
       </c>
       <c r="E73" s="15" t="inlineStr">
-        <is>
-          <t>Destansi</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="15" t="inlineStr">
-        <is>
-          <t>Cryo Burst</t>
-        </is>
-      </c>
-      <c r="B74" s="15" t="inlineStr">
-        <is>
-          <t>Yardimci</t>
-        </is>
-      </c>
-      <c r="C74" s="15" t="inlineStr">
-        <is>
-          <t>Slowed enemy: next hit deals +8 bonus damage</t>
-        </is>
-      </c>
-      <c r="D74" s="15" t="inlineStr">
-        <is>
-          <t>Yavasslatilmis dusmana sonraki vurus +8 bonus hasar</t>
-        </is>
-      </c>
-      <c r="E74" s="15" t="inlineStr">
-        <is>
-          <t>Ender</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="15" t="inlineStr">
-        <is>
-          <t>Arc Overload</t>
-        </is>
-      </c>
-      <c r="B75" s="15" t="inlineStr">
-        <is>
-          <t>Yardimci</t>
-        </is>
-      </c>
-      <c r="C75" s="15" t="inlineStr">
-        <is>
-          <t>Electrocute chain hits 2 additional enemies (5 damage each)</t>
-        </is>
-      </c>
-      <c r="D75" s="15" t="inlineStr">
-        <is>
-          <t>Electrocute zinciri 2 ek dusmana daha sicrar (5 hasar)</t>
-        </is>
-      </c>
-      <c r="E75" s="15" t="inlineStr">
         <is>
           <t>Ender</t>
         </is>

</xml_diff>